<commit_message>
[BattleUI] Battle/Turn Manager 구현과 전투씬 구현중
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/Character.xlsx
+++ b/JsonConverter/ExcelFiles/Character.xlsx
@@ -21,81 +21,99 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="39">
   <x:si>
+    <x:t>Id</x:t>
+  </x:si>
+  <x:si>
+    <x:t>헬레나</x:t>
+  </x:si>
+  <x:si>
+    <x:t>int</x:t>
+  </x:si>
+  <x:si>
+    <x:t>엘리</x:t>
+  </x:si>
+  <x:si>
+    <x:t>다니엘</x:t>
+  </x:si>
+  <x:si>
+    <x:t>빅토르</x:t>
+  </x:si>
+  <x:si>
+    <x:t>스킬</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BasicCostumeId</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_ellie</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Weapon_Sword_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>캐릭터 전체 컨셉이나 스토리</x:t>
+  </x:si>
+  <x:si>
+    <x:t>제발 뜻대로 움직여주라</x:t>
+  </x:si>
+  <x:si>
+    <x:t>최대Mp</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(name)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MaxMp</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MaxHp</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Name</x:t>
+  </x:si>
+  <x:si>
+    <x:t>string</x:t>
+  </x:si>
+  <x:si>
+    <x:t>최대Hp</x:t>
+  </x:si>
+  <x:si>
+    <x:t>skill_fireball_01,skill_normalSword_01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>skill_swing_01,skill_fireball_02,skill_explosion_01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Costume_03</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SkillList</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Description</x:t>
+  </x:si>
+  <x:si>
+    <x:t>잉여로운 버프 캐릭터</x:t>
+  </x:si>
+  <x:si>
+    <x:t>UseWeaponId</x:t>
+  </x:si>
+  <x:si>
+    <x:t>캐릭터 고유 ID</x:t>
+  </x:si>
+  <x:si>
     <x:t>IconPath</x:t>
   </x:si>
   <x:si>
-    <x:t>엘리</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Id</x:t>
-  </x:si>
-  <x:si>
-    <x:t>int</x:t>
-  </x:si>
-  <x:si>
-    <x:t>스킬</x:t>
-  </x:si>
-  <x:si>
-    <x:t>다니엘</x:t>
-  </x:si>
-  <x:si>
-    <x:t>헬레나</x:t>
-  </x:si>
-  <x:si>
-    <x:t>빅토르</x:t>
-  </x:si>
-  <x:si>
-    <x:t>skill_fireball_01,skill_normalSword_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MaxHp</x:t>
-  </x:si>
-  <x:si>
-    <x:t>최대Mp</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Name</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MaxMp</x:t>
-  </x:si>
-  <x:si>
-    <x:t>최대Hp</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(name)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>string</x:t>
-  </x:si>
-  <x:si>
-    <x:t>캐릭터 고유 ID</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Costume_03</x:t>
-  </x:si>
-  <x:si>
-    <x:t>잉여로운 버프 캐릭터</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SkillList</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Description</x:t>
-  </x:si>
-  <x:si>
-    <x:t>UseWeaponId</x:t>
+    <x:t>Weapon_Braclet_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>모든 마법을 사용할 수 있는 캐릭터</x:t>
   </x:si>
   <x:si>
     <x:t>소환 마법을 사용할 수 있는 캐릭터</x:t>
   </x:si>
   <x:si>
-    <x:t>Weapon_Braclet_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>모든 마법을 사용할 수 있는 캐릭터</x:t>
-  </x:si>
-  <x:si>
     <x:t>캐릭터 별로 무기가 고정인 경우용</x:t>
   </x:si>
   <x:si>
@@ -105,27 +123,12 @@
     <x:t>character_daniel_01</x:t>
   </x:si>
   <x:si>
+    <x:t>Weapon_CoffeeCup_1</x:t>
+  </x:si>
+  <x:si>
     <x:t>character_ellie_01</x:t>
   </x:si>
   <x:si>
-    <x:t>Weapon_CoffeeCup_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>skill_swing_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>제발 뜻대로 움직여주라</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BasicCostumeId</x:t>
-  </x:si>
-  <x:si>
-    <x:t>캐릭터 전체 컨셉이나 스토리</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Weapon_Sword_1</x:t>
-  </x:si>
-  <x:si>
     <x:t>skill_normalSword_01</x:t>
   </x:si>
   <x:si>
@@ -133,9 +136,6 @@
   </x:si>
   <x:si>
     <x:t>character_hellena_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_ellie</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -953,101 +953,101 @@
   <x:sheetData>
     <x:row r="1" spans="1:8" ht="15.75" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>16</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="B1" s="1"/>
       <x:c r="C1" s="1" t="s">
-        <x:v>33</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D1" s="2" t="s">
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="E1" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="G1" s="3" t="s">
-        <x:v>13</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="H1" s="3" t="s">
-        <x:v>10</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:9" ht="13.199999999999999">
       <x:c r="A2" s="1" t="s">
-        <x:v>14</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="B2" s="1" t="s">
-        <x:v>15</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C2" s="1" t="s">
-        <x:v>15</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="D2" s="1" t="s">
-        <x:v>15</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="E2" s="1" t="s">
-        <x:v>15</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="F2" s="1" t="s">
-        <x:v>15</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="G2" s="3" t="s">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H2" s="3" t="s">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I2" s="3" t="s">
-        <x:v>15</x:v>
+        <x:v>17</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:9" s="13" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A3" s="12" t="s">
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="B3" s="12" t="s">
-        <x:v>11</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C3" s="12" t="s">
-        <x:v>20</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="D3" s="14" t="s">
-        <x:v>19</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="E3" s="14" t="s">
-        <x:v>21</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F3" s="15" t="s">
-        <x:v>32</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G3" s="13" t="s">
-        <x:v>9</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="H3" s="13" t="s">
-        <x:v>12</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="I3" s="13" t="s">
-        <x:v>0</x:v>
+        <x:v>27</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:15" ht="15.75" customHeight="1">
       <x:c r="A4" s="4" t="s">
-        <x:v>37</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="B4" s="4" t="s">
-        <x:v>6</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C4" s="4" t="s">
-        <x:v>24</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="D4" s="5" t="s">
-        <x:v>8</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E4" s="5" t="s">
-        <x:v>23</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="F4" s="16" t="s">
-        <x:v>17</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="G4" s="5"/>
       <x:c r="H4" s="5"/>
@@ -1061,19 +1061,19 @@
     </x:row>
     <x:row r="5" spans="1:15" ht="15.75" customHeight="1">
       <x:c r="A5" s="4" t="s">
-        <x:v>26</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="B5" s="6" t="s">
-        <x:v>7</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C5" s="6" t="s">
-        <x:v>22</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="D5" s="5" t="s">
-        <x:v>35</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="E5" s="5" t="s">
-        <x:v>34</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="F5" s="5"/>
       <x:c r="G5" s="5"/>
@@ -1088,19 +1088,19 @@
     </x:row>
     <x:row r="6" spans="1:15" ht="15.75" customHeight="1">
       <x:c r="A6" s="6" t="s">
-        <x:v>27</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="B6" s="6" t="s">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C6" s="6" t="s">
-        <x:v>18</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="D6" s="5" t="s">
-        <x:v>36</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="E6" s="5" t="s">
-        <x:v>29</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="F6" s="5"/>
       <x:c r="G6" s="5"/>
@@ -1115,16 +1115,16 @@
     </x:row>
     <x:row r="7" spans="1:15" ht="15.75" customHeight="1">
       <x:c r="A7" s="4" t="s">
-        <x:v>28</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="B7" s="4" t="s">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C7" s="4" t="s">
-        <x:v>31</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D7" s="5" t="s">
-        <x:v>30</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E7" s="5"/>
       <x:c r="F7" s="5"/>
@@ -1135,7 +1135,7 @@
         <x:v>200</x:v>
       </x:c>
       <x:c r="I7" s="5" t="s">
-        <x:v>38</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="J7" s="5"/>
       <x:c r="K7" s="5"/>

</xml_diff>

<commit_message>
[버그수정] playerModel ==  null 인 버그 수정
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/Character.xlsx
+++ b/JsonConverter/ExcelFiles/Character.xlsx
@@ -21,121 +21,121 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="39">
   <x:si>
+    <x:t>최대Hp</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Name</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(name)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MaxHp</x:t>
+  </x:si>
+  <x:si>
+    <x:t>최대Mp</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MaxMp</x:t>
+  </x:si>
+  <x:si>
+    <x:t>string</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Weapon_Sword_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Icon/Icon_ellie</x:t>
+  </x:si>
+  <x:si>
+    <x:t>캐릭터 전체 컨셉이나 스토리</x:t>
+  </x:si>
+  <x:si>
+    <x:t>제발 뜻대로 움직여주라</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BasicCostumeId</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Weapon_Braclet_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>소환 마법을 사용할 수 있는 캐릭터</x:t>
+  </x:si>
+  <x:si>
+    <x:t>모든 마법을 사용할 수 있는 캐릭터</x:t>
+  </x:si>
+  <x:si>
+    <x:t>character_daniel_01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>캐릭터 별로 무기가 고정인 경우용</x:t>
+  </x:si>
+  <x:si>
+    <x:t>character_ellie_01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Weapon_CoffeeCup_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>character_victor_01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>다니엘</x:t>
+  </x:si>
+  <x:si>
     <x:t>Id</x:t>
   </x:si>
   <x:si>
+    <x:t>엘리</x:t>
+  </x:si>
+  <x:si>
     <x:t>헬레나</x:t>
   </x:si>
   <x:si>
+    <x:t>스킬</x:t>
+  </x:si>
+  <x:si>
     <x:t>int</x:t>
   </x:si>
   <x:si>
-    <x:t>엘리</x:t>
-  </x:si>
-  <x:si>
-    <x:t>다니엘</x:t>
-  </x:si>
-  <x:si>
     <x:t>빅토르</x:t>
   </x:si>
   <x:si>
-    <x:t>스킬</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BasicCostumeId</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Icon/Icon_ellie</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Weapon_Sword_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>캐릭터 전체 컨셉이나 스토리</x:t>
-  </x:si>
-  <x:si>
-    <x:t>제발 뜻대로 움직여주라</x:t>
-  </x:si>
-  <x:si>
-    <x:t>최대Mp</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(name)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MaxMp</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MaxHp</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Name</x:t>
-  </x:si>
-  <x:si>
-    <x:t>string</x:t>
-  </x:si>
-  <x:si>
-    <x:t>최대Hp</x:t>
+    <x:t>skill_rest_coffee_01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>skill_normalSword_01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>character_hellena_01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>UseWeaponId</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SkillList</x:t>
+  </x:si>
+  <x:si>
+    <x:t>잉여로운 버프 캐릭터</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Description</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Costume_03</x:t>
+  </x:si>
+  <x:si>
+    <x:t>캐릭터 고유 ID</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IconPath</x:t>
+  </x:si>
+  <x:si>
+    <x:t>skill_swing_01,skill_fireball_02,skill_explosion_01</x:t>
   </x:si>
   <x:si>
     <x:t>skill_fireball_01,skill_normalSword_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>skill_swing_01,skill_fireball_02,skill_explosion_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Costume_03</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SkillList</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Description</x:t>
-  </x:si>
-  <x:si>
-    <x:t>잉여로운 버프 캐릭터</x:t>
-  </x:si>
-  <x:si>
-    <x:t>UseWeaponId</x:t>
-  </x:si>
-  <x:si>
-    <x:t>캐릭터 고유 ID</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IconPath</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Weapon_Braclet_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>모든 마법을 사용할 수 있는 캐릭터</x:t>
-  </x:si>
-  <x:si>
-    <x:t>소환 마법을 사용할 수 있는 캐릭터</x:t>
-  </x:si>
-  <x:si>
-    <x:t>캐릭터 별로 무기가 고정인 경우용</x:t>
-  </x:si>
-  <x:si>
-    <x:t>character_victor_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>character_daniel_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Weapon_CoffeeCup_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>character_ellie_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>skill_normalSword_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>skill_rest_coffee_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>character_hellena_01</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -953,101 +953,101 @@
   <x:sheetData>
     <x:row r="1" spans="1:8" ht="15.75" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>26</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="B1" s="1"/>
       <x:c r="C1" s="1" t="s">
-        <x:v>10</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="D1" s="2" t="s">
-        <x:v>6</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="E1" s="2" t="s">
-        <x:v>31</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G1" s="3" t="s">
-        <x:v>18</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H1" s="3" t="s">
-        <x:v>12</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:9" ht="13.199999999999999">
       <x:c r="A2" s="1" t="s">
-        <x:v>13</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="B2" s="1" t="s">
-        <x:v>17</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C2" s="1" t="s">
-        <x:v>17</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D2" s="1" t="s">
-        <x:v>17</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="E2" s="1" t="s">
-        <x:v>17</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="F2" s="1" t="s">
-        <x:v>17</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G2" s="3" t="s">
-        <x:v>2</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="H2" s="3" t="s">
-        <x:v>2</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="I2" s="3" t="s">
-        <x:v>17</x:v>
+        <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:9" s="13" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A3" s="12" t="s">
-        <x:v>0</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="B3" s="12" t="s">
-        <x:v>16</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C3" s="12" t="s">
-        <x:v>23</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="D3" s="14" t="s">
-        <x:v>22</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="E3" s="14" t="s">
-        <x:v>25</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="F3" s="15" t="s">
-        <x:v>7</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="G3" s="13" t="s">
-        <x:v>15</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H3" s="13" t="s">
-        <x:v>14</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="I3" s="13" t="s">
-        <x:v>27</x:v>
+        <x:v>36</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:15" ht="15.75" customHeight="1">
       <x:c r="A4" s="4" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B4" s="4" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="C4" s="4" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="D4" s="5" t="s">
         <x:v>38</x:v>
       </x:c>
-      <x:c r="B4" s="4" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C4" s="4" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="D4" s="5" t="s">
-        <x:v>19</x:v>
-      </x:c>
       <x:c r="E4" s="5" t="s">
-        <x:v>28</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="F4" s="16" t="s">
-        <x:v>21</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="G4" s="5"/>
       <x:c r="H4" s="5"/>
@@ -1061,19 +1061,19 @@
     </x:row>
     <x:row r="5" spans="1:15" ht="15.75" customHeight="1">
       <x:c r="A5" s="4" t="s">
-        <x:v>32</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="B5" s="6" t="s">
-        <x:v>5</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C5" s="6" t="s">
-        <x:v>30</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="D5" s="5" t="s">
-        <x:v>36</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E5" s="5" t="s">
-        <x:v>9</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="F5" s="5"/>
       <x:c r="G5" s="5"/>
@@ -1088,19 +1088,19 @@
     </x:row>
     <x:row r="6" spans="1:15" ht="15.75" customHeight="1">
       <x:c r="A6" s="6" t="s">
-        <x:v>33</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="B6" s="6" t="s">
-        <x:v>4</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C6" s="6" t="s">
-        <x:v>24</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="D6" s="5" t="s">
-        <x:v>37</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="E6" s="5" t="s">
-        <x:v>34</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="F6" s="5"/>
       <x:c r="G6" s="5"/>
@@ -1115,16 +1115,16 @@
     </x:row>
     <x:row r="7" spans="1:15" ht="15.75" customHeight="1">
       <x:c r="A7" s="4" t="s">
-        <x:v>35</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B7" s="4" t="s">
-        <x:v>3</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C7" s="4" t="s">
-        <x:v>11</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D7" s="5" t="s">
-        <x:v>20</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="E7" s="5"/>
       <x:c r="F7" s="5"/>

</xml_diff>